<commit_message>
found a new way to use spacy for extracting areas
</commit_message>
<xml_diff>
--- a/Consolidated_Directory_v12_subset.xlsx
+++ b/Consolidated_Directory_v12_subset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C38354D-8943-4601-9815-C60A851277CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699A371A-3E6B-4087-83CE-E2805B3DB3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46185" yWindow="0" windowWidth="26010" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46200" yWindow="10440" windowWidth="25995" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="70">
   <si>
     <t>ID</t>
   </si>
@@ -131,39 +131,18 @@
     <t>United States</t>
   </si>
   <si>
-    <t>Williams</t>
-  </si>
-  <si>
-    <t>Aurora</t>
-  </si>
-  <si>
-    <t>Caroline</t>
-  </si>
-  <si>
     <t>New York</t>
   </si>
   <si>
     <t>Book of Negroes, British Headquarters Papers PRO 30/55/100; Loyalist evacuation shipping lists (1782–1784)</t>
   </si>
   <si>
-    <t>Philadelphia</t>
-  </si>
-  <si>
-    <t>Barber</t>
-  </si>
-  <si>
-    <t>Allen</t>
-  </si>
-  <si>
     <t>Arrival_Port</t>
   </si>
   <si>
     <t>Book One Part One</t>
   </si>
   <si>
-    <t>Ship Aurora bound for St. John's</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
@@ -173,82 +152,85 @@
     <t>Canada</t>
   </si>
   <si>
-    <t>47.5646794, -52.7066964</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>Richard Browne</t>
-  </si>
-  <si>
-    <t>James Moore</t>
-  </si>
-  <si>
     <t>Virginia</t>
   </si>
   <si>
-    <t>Billy</t>
-  </si>
-  <si>
-    <t>Billy Williams, 35, healthy stout man, (Richard Browne). Formerly lived with Mr. Moore of Reedy Island, Caroline, from whence he came with the 71st Regiment about 3 years ago.</t>
-  </si>
-  <si>
-    <t>Reedy Island</t>
-  </si>
-  <si>
-    <t>Rose</t>
-  </si>
-  <si>
-    <t>Richard</t>
-  </si>
-  <si>
-    <t>Rose Richard, 20, healthy young woman, (Thomas Richard). Property of Thomas Richard, a refugee from Philadelphia.</t>
+    <t>Ann</t>
   </si>
   <si>
     <t>Female</t>
   </si>
   <si>
-    <t>39.9527237, -75.1635262</t>
-  </si>
-  <si>
-    <t>Thomas Richard</t>
-  </si>
-  <si>
-    <t>Daniel</t>
-  </si>
-  <si>
-    <t>Daniel Barber, 70, worn out, (James Moore). Says he was made free by Mr. Austin Moore of little York nigh 20 years ago.</t>
-  </si>
-  <si>
-    <t>little York</t>
-  </si>
-  <si>
-    <t>41.0111483, -90.7462496</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Farmer</t>
-  </si>
-  <si>
-    <t>Sarah Farmer, 23, healthy young woman, (Mrs. Sharp).</t>
-  </si>
-  <si>
-    <t>Mrs. Sharp</t>
-  </si>
-  <si>
-    <t>Barbarry</t>
-  </si>
-  <si>
-    <t>Barbarry Allen, 22, healthy stout wench, (Humphry Winters). Property of Humphrey Winters of New York from Virginia.</t>
-  </si>
-  <si>
-    <t>37.5329655, -77.471394</t>
-  </si>
-  <si>
-    <t>Humphry Winters</t>
+    <t>Loyalist evacuation lists</t>
+  </si>
+  <si>
+    <t>Dinah</t>
+  </si>
+  <si>
+    <t>Jacob</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Peter</t>
+  </si>
+  <si>
+    <t>Pompey</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
+    <t>41.7962409, -71.5992372</t>
+  </si>
+  <si>
+    <t>Simmons</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Fall 1783</t>
+  </si>
+  <si>
+    <t>Wanton</t>
+  </si>
+  <si>
+    <t>St. John's River</t>
+  </si>
+  <si>
+    <t>38.0410576, -78.5055084</t>
+  </si>
+  <si>
+    <t>49.8613357, -97.1604127</t>
+  </si>
+  <si>
+    <t>Pompey Wanton, 25, squat fellow, B, (John Burgis). Formerly slave to Stephen Wanton, Rhode Island; left him at the Evacuation of said place. GBC.</t>
+  </si>
+  <si>
+    <t>Ann bound for St. John's River John Clark, Master</t>
+  </si>
+  <si>
+    <t>John Burgis</t>
+  </si>
+  <si>
+    <t>Stogdon</t>
+  </si>
+  <si>
+    <t>Peter Stogdon, 23, stout fellow, M, (James Scot). Formerly slave to Robert Stogdon, Princetown; left him about 3 years past. GBC.</t>
+  </si>
+  <si>
+    <t>James Scot</t>
+  </si>
+  <si>
+    <t>Jacob Smith, 20, stout fellow, B. Thomas Cropper of Accomack, Eastern Shore, Virginia, claimant. (James Scot). Formerly slave to Reuben Waterhouse near Horntown Eastern Shore, Virginia; left him summer 82 &amp; joined Capt. Kid in his whaleboat in the Chesepeake. GBC.</t>
+  </si>
+  <si>
+    <t>Dinah Simmons, 40, stout wench, M, (Peter FitzSimmons). Mr. FitzSimmons property as appears by a Bill of Sale produced.</t>
+  </si>
+  <si>
+    <t>Peter FitzSimmons</t>
   </si>
 </sst>
 </file>
@@ -588,45 +570,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG6"/>
+  <dimension ref="A1:AF5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="163.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="245.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="53.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="98.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="98.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="98.140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="1.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -682,78 +665,75 @@
         <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="T1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U1" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>754</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s">
         <v>44</v>
       </c>
-      <c r="W1" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="H2">
-        <v>1748</v>
+        <v>1758</v>
       </c>
       <c r="I2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J2" t="s">
         <v>32</v>
@@ -765,13 +745,13 @@
         <v>32</v>
       </c>
       <c r="M2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="N2" t="s">
         <v>34</v>
       </c>
       <c r="O2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -780,81 +760,78 @@
         <v>35</v>
       </c>
       <c r="R2" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="S2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T2" t="s">
+        <v>34</v>
+      </c>
+      <c r="U2" t="s">
+        <v>58</v>
+      </c>
+      <c r="V2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W2" t="s">
+        <v>34</v>
+      </c>
+      <c r="X2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>755</v>
+      </c>
+      <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="T2" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2">
-        <v>1783</v>
-      </c>
-      <c r="V2" t="s">
-        <v>48</v>
-      </c>
-      <c r="W2" t="s">
-        <v>49</v>
-      </c>
-      <c r="X2" t="s">
+      <c r="C3" t="s">
         <v>50</v>
       </c>
-      <c r="Y2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="D3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3">
+        <v>1760</v>
+      </c>
+      <c r="I3" t="s">
         <v>40</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H3">
-        <v>1763</v>
-      </c>
-      <c r="I3" t="s">
-        <v>61</v>
       </c>
       <c r="J3" t="s">
         <v>32</v>
@@ -866,7 +843,7 @@
         <v>32</v>
       </c>
       <c r="M3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="N3" t="s">
         <v>34</v>
@@ -881,81 +858,78 @@
         <v>35</v>
       </c>
       <c r="R3" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" t="s">
+        <v>56</v>
+      </c>
+      <c r="U3" t="s">
+        <v>58</v>
+      </c>
+      <c r="V3" t="s">
+        <v>42</v>
+      </c>
+      <c r="W3" t="s">
+        <v>60</v>
+      </c>
+      <c r="X3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>756</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
         <v>62</v>
       </c>
-      <c r="S3" t="s">
-        <v>39</v>
-      </c>
-      <c r="T3" t="s">
-        <v>39</v>
-      </c>
-      <c r="U3">
-        <v>1783</v>
-      </c>
-      <c r="V3" t="s">
-        <v>48</v>
-      </c>
-      <c r="W3" t="s">
-        <v>49</v>
-      </c>
-      <c r="X3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>63</v>
-      </c>
-      <c r="AF3" t="s">
+      <c r="H4">
+        <v>1763</v>
+      </c>
+      <c r="I4" t="s">
         <v>40</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4">
-        <v>1713</v>
-      </c>
-      <c r="I4" t="s">
-        <v>47</v>
       </c>
       <c r="J4" t="s">
         <v>32</v>
@@ -967,13 +941,13 @@
         <v>32</v>
       </c>
       <c r="M4" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="N4" t="s">
         <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="P4" t="s">
         <v>34</v>
@@ -982,81 +956,78 @@
         <v>35</v>
       </c>
       <c r="R4" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="S4" t="s">
+        <v>36</v>
+      </c>
+      <c r="T4" t="s">
+        <v>56</v>
+      </c>
+      <c r="U4" t="s">
+        <v>58</v>
+      </c>
+      <c r="V4" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" t="s">
+        <v>34</v>
+      </c>
+      <c r="X4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>757</v>
+      </c>
+      <c r="B5" t="s">
         <v>39</v>
       </c>
-      <c r="T4" t="s">
-        <v>39</v>
-      </c>
-      <c r="U4">
-        <v>1783</v>
-      </c>
-      <c r="V4" t="s">
-        <v>48</v>
-      </c>
-      <c r="W4" t="s">
-        <v>49</v>
-      </c>
-      <c r="X4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>53</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5">
+        <v>1743</v>
+      </c>
+      <c r="I5" t="s">
         <v>45</v>
-      </c>
-      <c r="C5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H5">
-        <v>1760</v>
-      </c>
-      <c r="I5" t="s">
-        <v>61</v>
       </c>
       <c r="J5" t="s">
         <v>32</v>
@@ -1086,22 +1057,22 @@
         <v>34</v>
       </c>
       <c r="S5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="T5" t="s">
-        <v>39</v>
-      </c>
-      <c r="U5">
-        <v>1783</v>
+        <v>56</v>
+      </c>
+      <c r="U5" t="s">
+        <v>58</v>
       </c>
       <c r="V5" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="W5" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="X5" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="Y5" t="s">
         <v>34</v>
@@ -1113,123 +1084,19 @@
         <v>34</v>
       </c>
       <c r="AB5" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="AC5" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="AD5" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="AE5" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="AF5" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" t="s">
         <v>46</v>
-      </c>
-      <c r="H6">
-        <v>1761</v>
-      </c>
-      <c r="I6" t="s">
-        <v>61</v>
-      </c>
-      <c r="J6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" t="s">
-        <v>33</v>
-      </c>
-      <c r="L6" t="s">
-        <v>32</v>
-      </c>
-      <c r="M6" t="s">
-        <v>39</v>
-      </c>
-      <c r="N6" t="s">
-        <v>34</v>
-      </c>
-      <c r="O6" t="s">
-        <v>54</v>
-      </c>
-      <c r="P6" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>35</v>
-      </c>
-      <c r="R6" t="s">
-        <v>74</v>
-      </c>
-      <c r="S6" t="s">
-        <v>39</v>
-      </c>
-      <c r="T6" t="s">
-        <v>39</v>
-      </c>
-      <c r="U6">
-        <v>1783</v>
-      </c>
-      <c r="V6" t="s">
-        <v>48</v>
-      </c>
-      <c r="W6" t="s">
-        <v>49</v>
-      </c>
-      <c r="X6" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>34</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AF6" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1352,7 +1219,7 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>